<commit_message>
Diseño de Persistencia v0.1
</commit_message>
<xml_diff>
--- a/WineApp/ReporteRankingVinos.xlsx
+++ b/WineApp/ReporteRankingVinos.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="50">
   <si>
     <t>Nombre del vino</t>
   </si>
@@ -41,112 +41,127 @@
     <t>Albariño Refrescante</t>
   </si>
   <si>
+    <t>790.0</t>
+  </si>
+  <si>
+    <t>La Estancia</t>
+  </si>
+  <si>
+    <t>Pedernal</t>
+  </si>
+  <si>
+    <t>San Juan</t>
+  </si>
+  <si>
+    <t>Argentina</t>
+  </si>
+  <si>
+    <t>4.9</t>
+  </si>
+  <si>
+    <t>Chardonnay</t>
+  </si>
+  <si>
     <t>Gewürztraminer Exótico</t>
   </si>
   <si>
+    <t>780.0</t>
+  </si>
+  <si>
     <t>Chardonnay Premium</t>
   </si>
   <si>
+    <t>750.0</t>
+  </si>
+  <si>
+    <t>4.8500004</t>
+  </si>
+  <si>
     <t>Carménère Suave</t>
   </si>
   <si>
+    <t>650.0</t>
+  </si>
+  <si>
+    <t>Las Rosas</t>
+  </si>
+  <si>
+    <t>San Rafael</t>
+  </si>
+  <si>
+    <t>Mendoza</t>
+  </si>
+  <si>
+    <t>4.8</t>
+  </si>
+  <si>
+    <t>Cabernet Sauvignon</t>
+  </si>
+  <si>
     <t>Sauvignon Blanc Fresco</t>
   </si>
   <si>
+    <t>710.0</t>
+  </si>
+  <si>
+    <t>Las Palmeras</t>
+  </si>
+  <si>
+    <t>Tulum Valley</t>
+  </si>
+  <si>
+    <t>Torrontés</t>
+  </si>
+  <si>
     <t>Malbec Reserva</t>
   </si>
   <si>
+    <t>500.0</t>
+  </si>
+  <si>
+    <t>Los Andes</t>
+  </si>
+  <si>
+    <t>Valle de Uco</t>
+  </si>
+  <si>
+    <t>4.766667</t>
+  </si>
+  <si>
+    <t>Malbec</t>
+  </si>
+  <si>
     <t>Cabernet Sauvignon Gran Reserva</t>
   </si>
   <si>
+    <t>600.0</t>
+  </si>
+  <si>
+    <t>4.75</t>
+  </si>
+  <si>
     <t>Zinfandel Intenso</t>
   </si>
   <si>
-    <t>790.0</t>
-  </si>
-  <si>
-    <t>780.0</t>
-  </si>
-  <si>
-    <t>750.0</t>
-  </si>
-  <si>
-    <t>650.0</t>
-  </si>
-  <si>
-    <t>710.0</t>
-  </si>
-  <si>
-    <t>500.0</t>
-  </si>
-  <si>
-    <t>600.0</t>
-  </si>
-  <si>
     <t>530.0</t>
   </si>
   <si>
-    <t>La Estancia</t>
-  </si>
-  <si>
-    <t>Las Rosas</t>
-  </si>
-  <si>
-    <t>Las Palmeras</t>
-  </si>
-  <si>
-    <t>Los Andes</t>
-  </si>
-  <si>
-    <t>Pedernal</t>
-  </si>
-  <si>
-    <t>San Rafael</t>
-  </si>
-  <si>
-    <t>Tulum Valley</t>
-  </si>
-  <si>
-    <t>Valle de Uco</t>
-  </si>
-  <si>
-    <t>San Juan</t>
-  </si>
-  <si>
-    <t>Mendoza</t>
-  </si>
-  <si>
-    <t>Argentina</t>
-  </si>
-  <si>
-    <t>4.9</t>
-  </si>
-  <si>
-    <t>4.8500004</t>
-  </si>
-  <si>
-    <t>4.8</t>
-  </si>
-  <si>
-    <t>4.766667</t>
-  </si>
-  <si>
-    <t>4.75</t>
-  </si>
-  <si>
     <t>4.7</t>
   </si>
   <si>
-    <t>Chardonnay</t>
-  </si>
-  <si>
-    <t>Cabernet Sauvignon</t>
-  </si>
-  <si>
-    <t>Torrontés</t>
-  </si>
-  <si>
-    <t>Malbec</t>
+    <t>Syrah Especial</t>
+  </si>
+  <si>
+    <t>520.0</t>
+  </si>
+  <si>
+    <t>Riesling Delicado</t>
+  </si>
+  <si>
+    <t>720.0</t>
+  </si>
+  <si>
+    <t>4.6</t>
   </si>
 </sst>
 </file>
@@ -191,8 +206,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
+  <cols>
+    <col min="1" max="1" width="31.41015625" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="10.60546875" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="20.3515625" customWidth="true" bestFit="true"/>
+    <col min="4" max="4" width="12.58203125" customWidth="true" bestFit="true"/>
+    <col min="5" max="5" width="9.40625" customWidth="true" bestFit="true"/>
+    <col min="6" max="6" width="9.81640625" customWidth="true" bestFit="true"/>
+    <col min="7" max="7" width="10.51171875" customWidth="true" bestFit="true"/>
+    <col min="8" max="8" width="18.9921875" customWidth="true" bestFit="true"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
@@ -254,178 +279,230 @@
         <v>17</v>
       </c>
       <c r="C3" t="s" s="0">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="D3" t="s" s="0">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="E3" t="s" s="0">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F3" t="s" s="0">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="G3" t="s" s="0">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="H3" t="s" s="0">
-        <v>23</v>
+        <v>15</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="0">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="B4" t="s" s="0">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="C4" t="s" s="0">
-        <v>24</v>
+        <v>10</v>
       </c>
       <c r="D4" t="s" s="0">
-        <v>25</v>
+        <v>11</v>
       </c>
       <c r="E4" t="s" s="0">
-        <v>26</v>
+        <v>12</v>
       </c>
       <c r="F4" t="s" s="0">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="G4" t="s" s="0">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="H4" t="s" s="0">
-        <v>27</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="B5" t="s" s="0">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="C5" t="s" s="0">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="D5" t="s" s="0">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="E5" t="s" s="0">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="F5" t="s" s="0">
-        <v>31</v>
+        <v>13</v>
       </c>
       <c r="G5" t="s" s="0">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="H5" t="s" s="0">
-        <v>31</v>
+        <v>27</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="B6" t="s" s="0">
+        <v>29</v>
+      </c>
+      <c r="C6" t="s" s="0">
+        <v>30</v>
+      </c>
+      <c r="D6" t="s" s="0">
+        <v>31</v>
+      </c>
+      <c r="E6" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="F6" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="G6" t="s" s="0">
+        <v>26</v>
+      </c>
+      <c r="H6" t="s" s="0">
         <v>32</v>
-      </c>
-      <c r="B6" t="s" s="0">
-        <v>32</v>
-      </c>
-      <c r="C6" t="s" s="0">
-        <v>32</v>
-      </c>
-      <c r="D6" t="s" s="0">
-        <v>33</v>
-      </c>
-      <c r="E6" t="s" s="0">
-        <v>32</v>
-      </c>
-      <c r="F6" t="s" s="0">
-        <v>33</v>
-      </c>
-      <c r="G6" t="s" s="0">
-        <v>33</v>
-      </c>
-      <c r="H6" t="s" s="0">
-        <v>33</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s" s="0">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B7" t="s" s="0">
         <v>34</v>
       </c>
       <c r="C7" t="s" s="0">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D7" t="s" s="0">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E7" t="s" s="0">
-        <v>34</v>
+        <v>25</v>
       </c>
       <c r="F7" t="s" s="0">
-        <v>34</v>
+        <v>13</v>
       </c>
       <c r="G7" t="s" s="0">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="H7" t="s" s="0">
-        <v>34</v>
+        <v>38</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s" s="0">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="B8" t="s" s="0">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="C8" t="s" s="0">
-        <v>36</v>
+        <v>23</v>
       </c>
       <c r="D8" t="s" s="0">
-        <v>37</v>
+        <v>24</v>
       </c>
       <c r="E8" t="s" s="0">
-        <v>37</v>
+        <v>25</v>
       </c>
       <c r="F8" t="s" s="0">
-        <v>38</v>
+        <v>13</v>
       </c>
       <c r="G8" t="s" s="0">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="H8" t="s" s="0">
-        <v>40</v>
+        <v>27</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s" s="0">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B9" t="s" s="0">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C9" t="s" s="0">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="D9" t="s" s="0">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="E9" t="s" s="0">
-        <v>43</v>
+        <v>25</v>
       </c>
       <c r="F9" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="G9" t="s" s="0">
         <v>44</v>
       </c>
-      <c r="G9" t="s" s="0">
-        <v>42</v>
-      </c>
       <c r="H9" t="s" s="0">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s" s="0">
+        <v>45</v>
+      </c>
+      <c r="B10" t="s" s="0">
+        <v>46</v>
+      </c>
+      <c r="C10" t="s" s="0">
+        <v>35</v>
+      </c>
+      <c r="D10" t="s" s="0">
+        <v>36</v>
+      </c>
+      <c r="E10" t="s" s="0">
+        <v>25</v>
+      </c>
+      <c r="F10" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="G10" t="s" s="0">
         <v>44</v>
+      </c>
+      <c r="H10" t="s" s="0">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s" s="0">
+        <v>47</v>
+      </c>
+      <c r="B11" t="s" s="0">
+        <v>48</v>
+      </c>
+      <c r="C11" t="s" s="0">
+        <v>30</v>
+      </c>
+      <c r="D11" t="s" s="0">
+        <v>31</v>
+      </c>
+      <c r="E11" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="F11" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="G11" t="s" s="0">
+        <v>49</v>
+      </c>
+      <c r="H11" t="s" s="0">
+        <v>32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>